<commit_message>
update to analysis script
</commit_message>
<xml_diff>
--- a/data/metric_types.xlsx
+++ b/data/metric_types.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zauner/Documents/Arbeit/12-TUM/MeLiDos/WP2.2.5_Data_Analysis/ZaunerEtAl_NatHumBehav_2026/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A48E0057-5F02-484B-8593-50BDD205EE4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A73CDE8-AD5F-C143-9875-464809B57D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16680" yWindow="4340" windowWidth="28240" windowHeight="17240" xr2:uid="{C7CE30F9-32C8-3B48-9C95-A21A5EBA7D2B}"/>
+    <workbookView xWindow="35300" yWindow="31100" windowWidth="28240" windowHeight="17240" xr2:uid="{C7CE30F9-32C8-3B48-9C95-A21A5EBA7D2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t>name</t>
   </si>
@@ -126,6 +126,15 @@
   </si>
   <si>
     <t>spectrum</t>
+  </si>
+  <si>
+    <t>metric_family</t>
+  </si>
+  <si>
+    <t>Interdaily stability</t>
+  </si>
+  <si>
+    <t>Intradaily variability</t>
   </si>
 </sst>
 </file>
@@ -167,10 +176,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -192,13 +200,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>101600</xdr:rowOff>
@@ -220,6 +228,1035 @@
       <xdr:spPr bwMode="auto">
         <a:xfrm>
           <a:off x="2476500" y="406400"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1025" name="AutoShape 1">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9A2FB98-7EE4-2F51-7AB6-3ABE8F8FD1DA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="406400"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1026" name="AutoShape 2">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DAFE5748-AA71-6425-307E-25108BD36B5C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="609600"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1027" name="AutoShape 3">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA854617-AFD5-0966-626A-F2F1210EA1DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="812800"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1028" name="AutoShape 4">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8AC6FDB2-8226-E46D-E300-0EC0E152A74D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="1016000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1029" name="AutoShape 5">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A232EEB6-1F38-4948-750F-68888077D75F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="1219200"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1030" name="AutoShape 6">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E6940D9-EB9B-A177-4141-56BB88E32B1A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="1422400"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1031" name="AutoShape 7">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA0C4C4D-AA50-14BD-995F-70F4A29DDF2D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="1625600"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1032" name="AutoShape 8">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{806A8F58-902B-7FEB-0372-7A6A0E625ED0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="1828800"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1033" name="AutoShape 9">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B014DAD5-E75B-E90D-7BAA-8B2B248E03F1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="2032000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1034" name="AutoShape 10">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9FEF192B-4E29-CCB5-D527-D5F84476AEB7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="2235200"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1035" name="AutoShape 11">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEEAB736-EB0C-DBF8-9EF3-94FA0C1BA32C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="2438400"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1036" name="AutoShape 12">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A7B3849-5698-D73E-BF90-C628B22C0E05}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="2641600"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1037" name="AutoShape 13">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{50775F31-7945-2D28-CBF2-11D637CF3ED2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="2844800"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1038" name="AutoShape 14">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E099BAF6-30AF-7269-9E0D-F7260CAFDD1E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="3048000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1039" name="AutoShape 15">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{516503E7-8AFB-30E0-C8C7-24F0DDFB0502}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="3251200"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1040" name="AutoShape 16">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9D8B835-DCC5-D9BE-AB95-4DA9EBAE9D24}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="3454400"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1041" name="AutoShape 17">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{22B25B04-46E4-090A-B99B-3EA593237C5F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="3657600"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1042" name="AutoShape 18">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C746CFC5-FCB9-0522-6223-F1C3EFD79411}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="3860800"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1043" name="AutoShape 19">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D795A655-769D-0725-4256-D701E535FC84}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="4064000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1044" name="AutoShape 20">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F80849BF-15A1-BB10-0BF0-121699EB6224}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="4267200"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1045" name="AutoShape 21">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30FED8C4-2EFA-B777-1BB4-DA0E82C70B10}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2679700" y="4470400"/>
           <a:ext cx="304800" cy="304800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -558,200 +1595,230 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A92DB5B6-BF99-7A49-82AC-8DE1D6829BB0}">
-  <dimension ref="A1:B23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A92DB5B6-BF99-7A49-82AC-8DE1D6829BB0}">
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" customWidth="1"/>
+    <col min="1" max="2" width="35.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1"/>
+      <c r="C7" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1"/>
+      <c r="C10" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1"/>
+      <c r="C11" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1"/>
+      <c r="C12" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1"/>
+      <c r="C15" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>